<commit_message>
fix: los asociados de ejemplo ingresan a laborar con al menos 18 años
La fecha de ingreso se sorteaba sin mirar la de nacimiento: 15 de los 50
asociados empezaban a trabajar siendo menores. Lo detectó el contrato de
datos (regla mayor_de_edad_al_ingreso). Se regenera data/ejemplo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ejemplo/asociados_ejemplo.xlsx
+++ b/data/ejemplo/asociados_ejemplo.xlsx
@@ -1199,7 +1199,7 @@
         <v>104</v>
       </c>
       <c r="AM3" s="1" t="n">
-        <v>35164</v>
+        <v>43199</v>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
         <v>106</v>
       </c>
       <c r="AM8" s="1" t="n">
-        <v>39209</v>
+        <v>41416</v>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
         <v>104</v>
       </c>
       <c r="AM10" s="1" t="n">
-        <v>38767</v>
+        <v>39748</v>
       </c>
       <c r="AN10" t="inlineStr">
         <is>
@@ -3291,7 +3291,7 @@
         <v>110</v>
       </c>
       <c r="AM11" s="1" t="n">
-        <v>35705</v>
+        <v>40107</v>
       </c>
       <c r="AN11" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
         <v>107</v>
       </c>
       <c r="AM14" s="1" t="n">
-        <v>38824</v>
+        <v>41698</v>
       </c>
       <c r="AN14" t="inlineStr">
         <is>
@@ -4867,7 +4867,7 @@
         <v>109</v>
       </c>
       <c r="AM17" s="1" t="n">
-        <v>39724</v>
+        <v>44797</v>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
@@ -5667,7 +5667,7 @@
         <v>107</v>
       </c>
       <c r="AM20" s="1" t="n">
-        <v>37488</v>
+        <v>43735</v>
       </c>
       <c r="AN20" t="inlineStr">
         <is>
@@ -6449,7 +6449,7 @@
         <v>107</v>
       </c>
       <c r="AM23" s="1" t="n">
-        <v>40972</v>
+        <v>44818</v>
       </c>
       <c r="AN23" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
         <v>107</v>
       </c>
       <c r="AM25" s="1" t="n">
-        <v>36290</v>
+        <v>38404</v>
       </c>
       <c r="AN25" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
         <v>109</v>
       </c>
       <c r="AM29" s="1" t="n">
-        <v>38002</v>
+        <v>43314</v>
       </c>
       <c r="AN29" t="inlineStr">
         <is>
@@ -8563,7 +8563,7 @@
         <v>101</v>
       </c>
       <c r="AM31" s="1" t="n">
-        <v>41033</v>
+        <v>43049</v>
       </c>
       <c r="AN31" t="inlineStr">
         <is>
@@ -10399,7 +10399,7 @@
         <v>109</v>
       </c>
       <c r="AM38" s="1" t="n">
-        <v>36430</v>
+        <v>40554</v>
       </c>
       <c r="AN38" t="inlineStr">
         <is>
@@ -12521,7 +12521,7 @@
         <v>101</v>
       </c>
       <c r="AM46" s="1" t="n">
-        <v>36117</v>
+        <v>44562</v>
       </c>
       <c r="AN46" t="inlineStr">
         <is>
@@ -12787,7 +12787,7 @@
         <v>101</v>
       </c>
       <c r="AM47" s="1" t="n">
-        <v>36006</v>
+        <v>42355</v>
       </c>
       <c r="AN47" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
         <v>107</v>
       </c>
       <c r="AM51" s="1" t="n">
-        <v>37747</v>
+        <v>38578</v>
       </c>
       <c r="AN51" t="inlineStr">
         <is>

</xml_diff>